<commit_message>
Update c++ pipeline and add new repos to excel
</commit_message>
<xml_diff>
--- a/PRs.xlsx
+++ b/PRs.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All PRs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New Repos" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11526,4 +11527,221 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Repo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>PR Number</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Algorithm Name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Paper Reference</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Has Test</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Test Links</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Has Benchmark</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Bench Links</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Has Issue</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>AI Generated</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>mdtraj/mdtraj</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2038</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>add formal charge in missing places on topology</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://github.com/mdtraj/mdtraj/pull/2038</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>fix_wrong_implementation</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Topology.join() formal charge propagation</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>tests/test_topology.py::test_topology_join_formal_charge</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Bug fix: formalCharge of metal ion is dropped when using Topology.join(); PR propagates the charge through copy() and add_atom().</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>rdkit/rdkit</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>8957</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Modern stereo: fix stereo inversion in rings</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://github.com/rdkit/rdkit/pull/8957</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>fix_wrong_implementation</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SMILES stereochemistry perception (CIP stereo in rings)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Code/GraphMol/catch_chirality.cpp</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Bug fix: modern stereo perception inverts atom parity in ring systems with multiple stereocenters; regression introduced by PR #8738 interacting with #1294.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>